<commit_message>
fix: dependent words counting fixed
</commit_message>
<xml_diff>
--- a/scripts/experementals/generic_tokens_expanded.xlsx
+++ b/scripts/experementals/generic_tokens_expanded.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rictus\IdeaProjects\tolstoy-words-local\scripts\experementals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D35626-E5AD-465E-A326-73FFD9BAD1B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA673C2C-9E37-4DD8-87BB-C54A1CC756CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2925" yWindow="2580" windowWidth="25815" windowHeight="11580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
   <si>
     <t>TokenID</t>
   </si>
@@ -86,6 +86,9 @@
   </si>
   <si>
     <t>VERB_HEAD</t>
+  </si>
+  <si>
+    <t>None</t>
   </si>
   <si>
     <t>запах</t>
@@ -556,19 +559,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V20"/>
+  <dimension ref="A1:W20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="18.5703125" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="17.7109375" customWidth="1"/>
-    <col min="5" max="5" width="24.85546875" customWidth="1"/>
-    <col min="6" max="6" width="19.5703125" customWidth="1"/>
-    <col min="7" max="7" width="21" customWidth="1"/>
-    <col min="22" max="22" width="17.42578125" customWidth="1"/>
+    <col min="4" max="4" width="26.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -635,16 +632,19 @@
       <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D2">
         <v>2331</v>
@@ -704,15 +704,15 @@
         <v>234</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D3">
         <v>1783</v>
@@ -769,15 +769,15 @@
         <v>193</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D4">
         <v>1115</v>
@@ -831,15 +831,15 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D5">
         <v>905</v>
@@ -881,15 +881,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6">
         <v>913</v>
@@ -946,15 +946,15 @@
         <v>130</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D7">
         <v>819</v>
@@ -1011,15 +1011,15 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D8">
         <v>642</v>
@@ -1073,15 +1073,15 @@
         <v>110</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9">
         <v>394</v>
@@ -1135,15 +1135,15 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D10">
         <v>367</v>
@@ -1200,15 +1200,15 @@
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D11">
         <v>192</v>
@@ -1256,15 +1256,15 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D12">
         <v>48</v>
@@ -1300,15 +1300,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D13">
         <v>44</v>
@@ -1353,15 +1353,15 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D14">
         <v>18</v>
@@ -1388,15 +1388,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D15">
         <v>12</v>
@@ -1423,15 +1423,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D16">
         <v>8</v>
@@ -1464,15 +1464,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D17">
         <v>3</v>
@@ -1502,15 +1502,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D18">
         <v>1</v>
@@ -1531,15 +1531,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" t="s">
         <v>56</v>
-      </c>
-      <c r="C19" t="s">
-        <v>55</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -1553,16 +1553,19 @@
       <c r="G19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="W19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C20" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D20">
         <v>1</v>

</xml_diff>